<commit_message>
add aggr_industry_6 to separate gov workers from ed/healthcare
- non education/healthcare government workers are now in aggr_industry_6 and aggr_industry_5 is all education/healthcare workers (including those that work for government)
- aggr_industry 1-4 remains the same and is made up of non-government workers
</commit_message>
<xml_diff>
--- a/examples/population_synthesizer/data/travel_survey_industry_crosswalk.xlsx
+++ b/examples/population_synthesizer/data/travel_survey_industry_crosswalk.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://psrcwa-my.sharepoint.com/personal/jkolberg_psrc_org/Documents/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JKolberg\PythonProjects\census_getter\examples\population_synthesizer\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="199" documentId="8_{03A76C6C-B57B-4FEA-AFCF-A4CAECA699AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{731039A9-3D33-441B-B1E6-5518E7334341}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61F67587-96FD-4F9F-AEB9-9026DE96795F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="19543" windowHeight="12377" xr2:uid="{47F308CA-0CA2-49B5-84C9-E130F48BF86E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{47F308CA-0CA2-49B5-84C9-E130F48BF86E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="90">
   <si>
     <t>Aggregated industries</t>
   </si>
@@ -77,15 +77,6 @@
     <t>df['C24070_022E'] + df['C24070_023E'] + df['C24070_024E'] + df['C24070_036E'] + df['C24070_037E'] + df['C24070_038E'] + df['C24070_050E'] + df['C24070_051E'] + df['C24070_052E'] + df['C24070_078E'] + df['C24070_079E'] + df['C24070_080E']</t>
   </si>
   <si>
-    <t>Government, healthcare, education</t>
-  </si>
-  <si>
-    <t>government, private healthcare/education</t>
-  </si>
-  <si>
-    <t>df['C24070_057E'] + df['C24070_025E'] + df['C24070_039E'] + df['C24070_053E'] + df['C24070_081E']</t>
-  </si>
-  <si>
     <t>ACS industries</t>
   </si>
   <si>
@@ -284,20 +275,44 @@
     <t xml:space="preserve">    Other Services (except Public Administration)</t>
   </si>
   <si>
-    <t xml:space="preserve">    Public Administration</t>
-  </si>
-  <si>
     <t>Class of worker: local, state, federal governemnt</t>
   </si>
   <si>
-    <t xml:space="preserve">All NAICS codes </t>
+    <t>df['C24070_025E'] + df['C24070_039E'] + df['C24070_053E'] + df['C24070_067E'] + df['C24070_081E']</t>
+  </si>
+  <si>
+    <t>df['C24070_058E'] + df['C24070_059E'] + df['C24070_060E'] + df['C24070_061E'] + df['C24070_062E'] + df['C24070_063E'] + df['C24070_064E'] + df['C24070_065E'] + df['C24070_066E'] + df['C24070_068E'] + df['C24070_069E'] + df['C24070_070E']</t>
+  </si>
+  <si>
+    <t>Government (exluding healthcare and education)</t>
+  </si>
+  <si>
+    <t>Healthcare, education</t>
+  </si>
+  <si>
+    <t>public/private healthcare/education</t>
+  </si>
+  <si>
+    <t>government</t>
+  </si>
+  <si>
+    <t>healthcare, education</t>
+  </si>
+  <si>
+    <t>Healthcare, Education</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    All other NAICS codes</t>
+  </si>
+  <si>
+    <t>11-92 (excluding 61-62)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -334,12 +349,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="2"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -674,31 +692,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FDC822C-DB23-4186-ADEB-84A80D26801D}">
-  <dimension ref="A1:D77"/>
-  <sheetFormatPr defaultRowHeight="14.65"/>
+  <dimension ref="A1:D79"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="56.140625" customWidth="1"/>
-    <col min="2" max="2" width="67.5703125" customWidth="1"/>
+    <col min="1" max="1" width="56.109375" customWidth="1"/>
+    <col min="2" max="2" width="67.5546875" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="24.28515625" customWidth="1"/>
-    <col min="5" max="5" width="36.7109375" customWidth="1"/>
+    <col min="4" max="4" width="24.33203125" customWidth="1"/>
+    <col min="5" max="5" width="36.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -712,7 +730,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -726,7 +744,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -740,7 +758,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -754,31 +772,45 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>83</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>84</v>
       </c>
       <c r="C6">
         <v>5</v>
       </c>
       <c r="D6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>82</v>
+      </c>
+      <c r="B7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C7">
+        <v>6</v>
+      </c>
+      <c r="D7" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
         <v>15</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="1" t="s">
-        <v>18</v>
       </c>
       <c r="B11" t="s">
         <v>4</v>
@@ -787,9 +819,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B12" t="s">
         <v>4</v>
@@ -798,9 +830,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B13" t="s">
         <v>7</v>
@@ -809,9 +841,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B14" t="s">
         <v>7</v>
@@ -820,9 +852,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B15" t="s">
         <v>9</v>
@@ -831,9 +863,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B16" t="s">
         <v>7</v>
@@ -842,9 +874,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B17" t="s">
         <v>11</v>
@@ -853,9 +885,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B18" t="s">
         <v>11</v>
@@ -864,9 +896,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B19" t="s">
         <v>11</v>
@@ -875,20 +907,20 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>13</v>
+        <v>86</v>
       </c>
       <c r="C20">
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B21" t="s">
         <v>9</v>
@@ -897,9 +929,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B22" t="s">
         <v>9</v>
@@ -908,133 +940,133 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B23" t="s">
+        <v>36</v>
+      </c>
+      <c r="C23">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="1"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" t="s">
         <v>30</v>
       </c>
-      <c r="B23" t="s">
-        <v>13</v>
-      </c>
-      <c r="C23">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3">
-      <c r="A24" s="1"/>
-    </row>
-    <row r="26" spans="1:3">
-      <c r="A26" s="2" t="s">
+      <c r="C27">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
         <v>31</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C26" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="A27" t="s">
+      <c r="B28" t="s">
         <v>32</v>
-      </c>
-      <c r="B27" t="s">
-        <v>33</v>
-      </c>
-      <c r="C27">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3">
-      <c r="A28" t="s">
-        <v>34</v>
-      </c>
-      <c r="B28" t="s">
-        <v>35</v>
       </c>
       <c r="C28">
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:3">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B29" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C29">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:3">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
+        <v>34</v>
+      </c>
+      <c r="B30" t="s">
+        <v>35</v>
+      </c>
+      <c r="C30">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" t="s">
+        <v>36</v>
+      </c>
+      <c r="C31">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
         <v>37</v>
       </c>
-      <c r="B30" t="s">
-        <v>38</v>
-      </c>
-      <c r="C30">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3">
-      <c r="A31" t="s">
-        <v>39</v>
-      </c>
-      <c r="B31" t="s">
-        <v>35</v>
-      </c>
-      <c r="C31">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3">
-      <c r="A32" t="s">
-        <v>40</v>
-      </c>
       <c r="B32" t="s">
-        <v>35</v>
+        <v>87</v>
       </c>
       <c r="C32">
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:3">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>38</v>
+      </c>
+      <c r="B33" t="s">
+        <v>30</v>
+      </c>
+      <c r="C33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>39</v>
+      </c>
+      <c r="B34" t="s">
+        <v>40</v>
+      </c>
+      <c r="C34">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
         <v>41</v>
       </c>
-      <c r="B33" t="s">
-        <v>33</v>
-      </c>
-      <c r="C33">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3">
-      <c r="A34" t="s">
+      <c r="B35" t="s">
         <v>42</v>
-      </c>
-      <c r="B34" t="s">
-        <v>43</v>
-      </c>
-      <c r="C34">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3">
-      <c r="A35" t="s">
-        <v>44</v>
-      </c>
-      <c r="B35" t="s">
-        <v>45</v>
       </c>
       <c r="C35">
         <v>2</v>
       </c>
     </row>
-    <row r="36" spans="1:3">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B36" t="s">
         <v>11</v>
@@ -1043,157 +1075,157 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="1:3">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B37" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C37">
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:3">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B38" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C38">
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:3">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B39" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C39">
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:3">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B40" t="s">
-        <v>35</v>
+        <v>87</v>
       </c>
       <c r="C40">
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:3">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B41" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C41">
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="1:3">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B42" t="s">
-        <v>35</v>
+        <v>87</v>
       </c>
       <c r="C42">
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:3">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B43" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C43">
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:3">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B44" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C44">
         <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:3">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B45" t="s">
-        <v>35</v>
+        <v>87</v>
       </c>
       <c r="C45">
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:3">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B46" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C46">
         <v>3</v>
       </c>
     </row>
-    <row r="47" spans="1:3">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B47" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C47">
         <v>4</v>
       </c>
     </row>
-    <row r="48" spans="1:3">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B48" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="C48">
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:3">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
         <v>59</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3">
-      <c r="A52" t="s">
-        <v>60</v>
-      </c>
-      <c r="B52" t="s">
-        <v>61</v>
-      </c>
-      <c r="C52" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3">
-      <c r="A53" t="s">
-        <v>62</v>
       </c>
       <c r="B53">
         <v>11</v>
@@ -1202,9 +1234,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:3">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B54">
         <v>21</v>
@@ -1213,9 +1245,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:3">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B55">
         <v>22</v>
@@ -1224,9 +1256,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:3">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B56">
         <v>23</v>
@@ -1235,9 +1267,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="57" spans="1:3">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B57">
         <v>31</v>
@@ -1246,9 +1278,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="58" spans="1:3">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B58">
         <v>32</v>
@@ -1257,9 +1289,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="1:3">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B59">
         <v>33</v>
@@ -1268,9 +1300,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="1:3">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B60">
         <v>42</v>
@@ -1279,9 +1311,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="1:3">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B61">
         <v>44</v>
@@ -1290,9 +1322,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="62" spans="1:3">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B62">
         <v>45</v>
@@ -1301,9 +1333,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="63" spans="1:3">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B63">
         <v>48</v>
@@ -1312,9 +1344,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="64" spans="1:3">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B64">
         <v>49</v>
@@ -1323,9 +1355,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="1:3">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B65">
         <v>51</v>
@@ -1334,9 +1366,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="66" spans="1:3">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B66">
         <v>52</v>
@@ -1345,9 +1377,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:3">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B67">
         <v>53</v>
@@ -1356,9 +1388,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="68" spans="1:3">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B68">
         <v>54</v>
@@ -1367,9 +1399,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="69" spans="1:3">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B69">
         <v>55</v>
@@ -1378,9 +1410,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="70" spans="1:3">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B70">
         <v>56</v>
@@ -1389,9 +1421,9 @@
         <v>4</v>
       </c>
     </row>
-    <row r="71" spans="1:3">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B71">
         <v>61</v>
@@ -1400,9 +1432,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="72" spans="1:3">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B72">
         <v>62</v>
@@ -1411,9 +1443,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="73" spans="1:3">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B73">
         <v>71</v>
@@ -1422,9 +1454,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="74" spans="1:3">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B74">
         <v>72</v>
@@ -1433,9 +1465,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:3">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B75">
         <v>81</v>
@@ -1444,26 +1476,42 @@
         <v>3</v>
       </c>
     </row>
-    <row r="76" spans="1:3">
-      <c r="A76" t="s">
-        <v>82</v>
-      </c>
-      <c r="B76">
-        <v>92</v>
-      </c>
-      <c r="C76">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A76" s="2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>83</v>
-      </c>
-      <c r="B77" t="s">
-        <v>84</v>
+        <v>74</v>
+      </c>
+      <c r="B77">
+        <v>61</v>
       </c>
       <c r="C77">
         <v>5</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>75</v>
+      </c>
+      <c r="B78">
+        <v>62</v>
+      </c>
+      <c r="C78">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>88</v>
+      </c>
+      <c r="B79" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C79">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>